<commit_message>
fixed platetype flowing to transfer list
</commit_message>
<xml_diff>
--- a/public/data/RippleTemplate_Combinator.xlsx
+++ b/public/data/RippleTemplate_Combinator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adalecki\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\adalecki\Projects\react\ripple\dist\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0047C85E-8723-49CF-826A-8C180A9E0705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2ECBE5C-F52C-4BC9-99CB-7452347B5E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-13365" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{EB7423B8-AA85-4736-B962-C2AEBC627853}"/>
+    <workbookView xWindow="28680" yWindow="-13365" windowWidth="38640" windowHeight="21120" xr2:uid="{EB7423B8-AA85-4736-B962-C2AEBC627853}"/>
   </bookViews>
   <sheets>
     <sheet name="Patterns" sheetId="1" r:id="rId1"/>
@@ -187,60 +187,6 @@
     <t>E02</t>
   </si>
   <si>
-    <t>H2Aa</t>
-  </si>
-  <si>
-    <t>H2Ab</t>
-  </si>
-  <si>
-    <t>H2Ac</t>
-  </si>
-  <si>
-    <t>H2Ad</t>
-  </si>
-  <si>
-    <t>H2Ba</t>
-  </si>
-  <si>
-    <t>H2Bb</t>
-  </si>
-  <si>
-    <t>H2Bc</t>
-  </si>
-  <si>
-    <t>H2Bd</t>
-  </si>
-  <si>
-    <t>H3a</t>
-  </si>
-  <si>
-    <t>H3b</t>
-  </si>
-  <si>
-    <t>H3c</t>
-  </si>
-  <si>
-    <t>H3d</t>
-  </si>
-  <si>
-    <t>H4a</t>
-  </si>
-  <si>
-    <t>H4b</t>
-  </si>
-  <si>
-    <t>H4c</t>
-  </si>
-  <si>
-    <t>H4d</t>
-  </si>
-  <si>
-    <t>DNA1</t>
-  </si>
-  <si>
-    <t>DNA2</t>
-  </si>
-  <si>
     <t>SrcPlt1</t>
   </si>
   <si>
@@ -266,6 +212,60 @@
   </si>
   <si>
     <t>A06:P09</t>
+  </si>
+  <si>
+    <t>Comp1v1</t>
+  </si>
+  <si>
+    <t>Comp1v2</t>
+  </si>
+  <si>
+    <t>Comp1v3</t>
+  </si>
+  <si>
+    <t>Comp1v4</t>
+  </si>
+  <si>
+    <t>Comp2v1</t>
+  </si>
+  <si>
+    <t>Comp2v2</t>
+  </si>
+  <si>
+    <t>Comp2v3</t>
+  </si>
+  <si>
+    <t>Comp2v4</t>
+  </si>
+  <si>
+    <t>Comp3v1</t>
+  </si>
+  <si>
+    <t>Comp3v2</t>
+  </si>
+  <si>
+    <t>Comp3v3</t>
+  </si>
+  <si>
+    <t>Comp3v4</t>
+  </si>
+  <si>
+    <t>Comp4v2</t>
+  </si>
+  <si>
+    <t>Comp4v1</t>
+  </si>
+  <si>
+    <t>Comp4v3</t>
+  </si>
+  <si>
+    <t>Comp4v4</t>
+  </si>
+  <si>
+    <t>Comp5v1</t>
+  </si>
+  <si>
+    <t>Comp5v2</t>
   </si>
 </sst>
 </file>
@@ -712,13 +712,13 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="D3">
         <v>50</v>
@@ -772,330 +772,330 @@
         <v>29</v>
       </c>
       <c r="E1" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
         <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="D2">
         <v>50</v>
       </c>
       <c r="E2" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
         <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D3">
         <v>50</v>
       </c>
       <c r="E3" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B4" t="s">
         <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="D4">
         <v>50</v>
       </c>
       <c r="E4" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
         <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D5">
         <v>50</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
         <v>34</v>
       </c>
       <c r="C6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6">
+        <v>50</v>
+      </c>
+      <c r="E6" t="s">
         <v>52</v>
-      </c>
-      <c r="D6">
-        <v>50</v>
-      </c>
-      <c r="E6" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
         <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D7">
         <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
         <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D8">
         <v>50</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
         <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D9">
         <v>50</v>
       </c>
       <c r="E9" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
         <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="D10">
         <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B11" t="s">
         <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="D11">
         <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B12" t="s">
         <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D12">
         <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
         <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="D13">
         <v>50</v>
       </c>
       <c r="E13" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
         <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="D14">
         <v>50</v>
       </c>
       <c r="E14" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B15" t="s">
         <v>43</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="D15">
         <v>50</v>
       </c>
       <c r="E15" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
         <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D16">
         <v>50</v>
       </c>
       <c r="E16" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
         <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D17">
         <v>50</v>
       </c>
       <c r="E17" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="B18" t="s">
         <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="D18">
         <v>50</v>
       </c>
       <c r="E18" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="B19" t="s">
         <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="D19">
         <v>50</v>
       </c>
       <c r="E19" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="B20" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="D20">
         <v>50</v>
       </c>
       <c r="E20" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1148,22 +1148,22 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1171,22 +1171,22 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F3" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G3" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1194,22 +1194,22 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F4" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G4" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -1217,22 +1217,22 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F5" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G5" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1240,22 +1240,22 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E6" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G6" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -1263,22 +1263,22 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D7" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F7" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G7" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1286,22 +1286,22 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D8" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F8" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G8" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1309,22 +1309,22 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F9" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G9" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1332,22 +1332,22 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F10" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G10" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1355,22 +1355,22 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F11" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G11" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1378,22 +1378,22 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E12" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G12" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -1401,22 +1401,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E13" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G13" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1424,22 +1424,22 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D14" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E14" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F14" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G14" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1447,22 +1447,22 @@
         <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D15" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E15" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F15" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G15" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1470,22 +1470,22 @@
         <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D16" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E16" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F16" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G16" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1493,22 +1493,22 @@
         <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F17" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G17" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1516,22 +1516,22 @@
         <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C18" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E18" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F18" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G18" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1539,22 +1539,22 @@
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="C19" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E19" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F19" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G19" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1562,22 +1562,22 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D20" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E20" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F20" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G20" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1585,22 +1585,22 @@
         <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D21" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E21" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F21" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G21" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1608,22 +1608,22 @@
         <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C22" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D22" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E22" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F22" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G22" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1631,22 +1631,22 @@
         <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D23" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E23" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F23" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G23" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1654,22 +1654,22 @@
         <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C24" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E24" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F24" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G24" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1677,22 +1677,22 @@
         <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C25" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D25" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E25" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F25" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G25" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1700,22 +1700,22 @@
         <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C26" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D26" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E26" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F26" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G26" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1723,22 +1723,22 @@
         <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C27" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E27" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F27" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G27" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1746,22 +1746,22 @@
         <v>12</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C28" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D28" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E28" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F28" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G28" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1769,22 +1769,22 @@
         <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C29" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D29" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E29" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F29" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G29" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1792,22 +1792,22 @@
         <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C30" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D30" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E30" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F30" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G30" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1815,22 +1815,22 @@
         <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C31" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D31" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E31" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F31" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G31" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1838,22 +1838,22 @@
         <v>12</v>
       </c>
       <c r="B32" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C32" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D32" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E32" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F32" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G32" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -1861,758 +1861,758 @@
         <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="C33" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D33" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E33" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F33" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G33" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B34" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C34" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D34" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E34" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F34" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G34" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B35" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="C35" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D35" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E35" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F35" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G35" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B36" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C36" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D36" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E36" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F36" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G36" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B37" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C37" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D37" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E37" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F37" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G37" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C38" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D38" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E38" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F38" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G38" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B39" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C39" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D39" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E39" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F39" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G39" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B40" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C40" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D40" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E40" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F40" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G40" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B41" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C41" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D41" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E41" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F41" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G41" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B42" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C42" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D42" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E42" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F42" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G42" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B43" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C43" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D43" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E43" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F43" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G43" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C44" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D44" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E44" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F44" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G44" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B45" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C45" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D45" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E45" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F45" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G45" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>54</v>
+      </c>
+      <c r="B46" t="s">
+        <v>57</v>
+      </c>
+      <c r="C46" t="s">
+        <v>61</v>
+      </c>
+      <c r="D46" t="s">
+        <v>65</v>
+      </c>
+      <c r="E46" t="s">
         <v>72</v>
       </c>
-      <c r="B46" t="s">
-        <v>48</v>
-      </c>
-      <c r="C46" t="s">
-        <v>52</v>
-      </c>
-      <c r="D46" t="s">
-        <v>56</v>
-      </c>
-      <c r="E46" t="s">
-        <v>63</v>
-      </c>
       <c r="F46" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G46" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>54</v>
+      </c>
+      <c r="B47" t="s">
+        <v>60</v>
+      </c>
+      <c r="C47" t="s">
+        <v>64</v>
+      </c>
+      <c r="D47" t="s">
+        <v>68</v>
+      </c>
+      <c r="E47" t="s">
         <v>72</v>
       </c>
-      <c r="B47" t="s">
-        <v>51</v>
-      </c>
-      <c r="C47" t="s">
-        <v>55</v>
-      </c>
-      <c r="D47" t="s">
-        <v>59</v>
-      </c>
-      <c r="E47" t="s">
-        <v>63</v>
-      </c>
       <c r="F47" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G47" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B48" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C48" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D48" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E48" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F48" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G48" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B49" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="C49" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D49" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E49" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F49" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G49" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B50" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C50" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D50" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E50" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F50" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G50" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B51" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="C51" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D51" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E51" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F51" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G51" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B52" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C52" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D52" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E52" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F52" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G52" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C53" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D53" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E53" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F53" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G53" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B54" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C54" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D54" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E54" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F54" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G54" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C55" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D55" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E55" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F55" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G55" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C56" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D56" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E56" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F56" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G56" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B57" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C57" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D57" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E57" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F57" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G57" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B58" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C58" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D58" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E58" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F58" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G58" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B59" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C59" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D59" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E59" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F59" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G59" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B60" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C60" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D60" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E60" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F60" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G60" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B61" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C61" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D61" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E61" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F61" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G61" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>54</v>
+      </c>
+      <c r="B62" t="s">
+        <v>57</v>
+      </c>
+      <c r="C62" t="s">
+        <v>61</v>
+      </c>
+      <c r="D62" t="s">
+        <v>65</v>
+      </c>
+      <c r="E62" t="s">
         <v>72</v>
       </c>
-      <c r="B62" t="s">
-        <v>48</v>
-      </c>
-      <c r="C62" t="s">
-        <v>52</v>
-      </c>
-      <c r="D62" t="s">
-        <v>56</v>
-      </c>
-      <c r="E62" t="s">
-        <v>63</v>
-      </c>
       <c r="F62" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G62" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>54</v>
+      </c>
+      <c r="B63" t="s">
+        <v>60</v>
+      </c>
+      <c r="C63" t="s">
+        <v>64</v>
+      </c>
+      <c r="D63" t="s">
+        <v>68</v>
+      </c>
+      <c r="E63" t="s">
         <v>72</v>
       </c>
-      <c r="B63" t="s">
-        <v>51</v>
-      </c>
-      <c r="C63" t="s">
-        <v>55</v>
-      </c>
-      <c r="D63" t="s">
-        <v>59</v>
-      </c>
-      <c r="E63" t="s">
-        <v>63</v>
-      </c>
       <c r="F63" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G63" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B64" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C64" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D64" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E64" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F64" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G64" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B65" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="C65" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D65" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E65" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F65" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G65" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>